<commit_message>
Add Texas advisor-level pass: 36 named people across 9 banks
Second pass over the confirmed Texas programs, taking the state from 5
named people to 36. New "Texas Advisors" tab in the workbook plus a
companion markdown roster.

Best finds: ANBTX published a full 7-person trust roster with direct
dials and emails; Prosperity's program is a manager plus nine advisors
at $600MM+ under Randy Hall; Texas Regional Bank just hired a CIO into
a brand-new division; Woodforest brought in an advisor managing ~$197MM
in Aug 2024.

Correction: First Financial runs TWO channels, not in-house trust only.
It also has First Financial Investment Advisors on Raymond James.
Platform summary updated accordingly.

No CRD was captured for any Texas advisor and no registration is
verified — FINRA, SEC IAPD and FDIC remain blocked from this
environment.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012NtTkX4kFFRh2WeKuPwqNf
</commit_message>
<xml_diff>
--- a/texas-banks-wealth-management.xlsx
+++ b/texas-banks-wealth-management.xlsx
@@ -8,10 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tier 1 - Texas HQ Banks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tier 2 - Out of State" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Texas Advisors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tier 1 - Texas HQ Banks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tier 2 - Out of State" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Texas Advisors'!$A$4:$I$40</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -116,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -135,6 +138,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -500,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -520,6 +524,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -537,7 +542,7 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>It is NOT an advisor-level pass. Only five individual names surfaced across the whole state. Every program here needs a second pass to become callable.</t>
+          <t>SUPERSEDED: an advisor-level pass on 2026-09-07 raised this from 5 names to 36 across 9 banks. See the Texas Advisors tab.</t>
         </is>
       </c>
     </row>
@@ -555,6 +560,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -590,6 +596,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -625,6 +632,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -667,12 +675,1616 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="72" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Texas Bank Advisors — named people by bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>36 named people across 9 banks. NO CRD captured for any Texas advisor and no registration verified — FINRA was unreachable. Run BrokerCheck before calling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Title / Role</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Direct phone</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Why this person</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>American National Bank of TX</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Elisa Luque</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Director of Wealth Management</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Terrell / N. Texas</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>elisaluque@anbtx.com</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>ENTRY POINT for the whole division. 13th largest trust org in Texas, $3B+ AUM.</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>https://www.anbtx.com/wealth-management/trust-professionals/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>American National Bank of TX</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Justin Fruhwirth</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>VP, Senior Portfolio Manager</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Terrell / N. Texas</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>214.863.6944</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>justinfruhwirth@anbtx.com</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>THE MODEL BUYER. He selects holdings, not just relationships.</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>https://www.anbtx.com/wealth-management/trust-professionals/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>American National Bank of TX</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Vickie Gutierrez</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>VP, Trust Officer</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Terrell / N. Texas</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>214.863.6548</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>vickiegutierrez@anbtx.com</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>https://www.anbtx.com/wealth-management/trust-professionals/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>American National Bank of TX</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Seth Jungman</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>VP, Trust Officer</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Terrell / N. Texas</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>214.863.6075</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>sethjungman@anbtx.com</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr"/>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>https://www.anbtx.com/wealth-management/trust-professionals/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>American National Bank of TX</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Margaret Svoboda</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>VP, Trust Officer</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Terrell / N. Texas</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>214.863.6801</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>margaretsvoboda@anbtx.com</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>https://www.anbtx.com/wealth-management/trust-professionals/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>American National Bank of TX</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Keely Johnson</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>AVP, Trust Officer</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Terrell / N. Texas</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>214.863.6077</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>keelyjohnson@anbtx.com</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr"/>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>https://www.anbtx.com/wealth-management/trust-professionals/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>American National Bank of TX</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Christie McKee</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>AVP, Trust Officer</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Terrell / N. Texas</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>214.863.6076</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>christiemckee@anbtx.com</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr"/>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>https://www.anbtx.com/wealth-management/trust-professionals/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Prosperity Bank</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Randy Hall</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Senior VP and Program Manager</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Victoria TX (program HQ)</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>r***@prosperitybankusa.com</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Raymond James Fin. Svcs</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>ONE CALL OPENS NINE ADVISORS and $600MM+ across Texas and Oklahoma.</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>https://www.prosperitybankusa.com/prosperityprivate-investments-bios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Prosperity Bank</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Michael Hanson</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Senior Financial Advisor (RJ Dallas branch)</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Raymond James Fin. Svcs</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Covers 16 branches across DFW and East Texas on his own.</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>https://www.prosperitybankusa.com/prosperityprivate-investments-bios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Prosperity Bank</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Felicia Brightbill</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Financial Advisor</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Lubbock</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Raymond James Fin. Svcs</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>West Texas territory.</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>https://www.prosperitybankusa.com/prosperityprivate-investments-bios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Prosperity Bank</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Brad (surname not found)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Financial Advisor</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Raymond James Fin. Svcs</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>25+ years, joined the program in 2005.</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>https://www.prosperitybankusa.com/prosperityprivate-investments-bios/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Woodforest National Bank</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Steve Tucker</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>President, Woodforest Wealth Strategies</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>The Woodlands</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Raymond James Fin. Svcs</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Program-level decision maker. Advisors sit in 7 bank offices across greater Houston.</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>https://www.raymondjames.com/woodforestadvisors/about-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Woodforest National Bank</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Ronald Folwell</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Financial Advisor</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>The Woodlands</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Raymond James Fin. Svcs</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Joined Aug 2024 from United Capital MANAGING ~$197MM. Recent enough that he is likely still building.</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>https://www.raymondjames.com/woodforestadvisors/about-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Woodforest National Bank</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Jonathan Murdock, CFP, CPWA</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Vice President</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>The Woodlands</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Raymond James Fin. Svcs</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>CPWA marks him as the high-net-worth specialist.</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>https://www.raymondjames.com/woodforestadvisors/about-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Woodforest National Bank</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Laura Folwell</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Client Services Coordinator</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>The Woodlands</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr"/>
+      <c r="F19" s="7" t="inlineStr"/>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Raymond James Fin. Svcs</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Gatekeeper.</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>https://www.raymondjames.com/woodforestadvisors/about-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Woodforest National Bank</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Heather Bucharski</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Client Service Associate</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>The Woodlands</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr"/>
+      <c r="F20" s="7" t="inlineStr"/>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Raymond James Fin. Svcs</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr"/>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>https://www.raymondjames.com/woodforestadvisors/about-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Texas Capital Bank</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Jim Brown</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Managing Director, Senior INVESTMENT Advisor</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr"/>
+      <c r="F21" s="7" t="inlineStr"/>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Own SEC-registered RIA</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>START HERE at this bank. Builds custom portfolios for individuals, family offices and institutions. The others are relationship-side.</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>https://texascapitalbank.com/private-bank/meet-our-advisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Texas Capital Bank</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Rob Ball</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Managing Director, Senior Private Client Advisor</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+      <c r="F22" s="7" t="inlineStr"/>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Own SEC-registered RIA</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Wealth advisory, investment mgmt, custom credit, personal trust, concierge private banking.</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>https://texascapitalbank.com/private-bank/meet-our-advisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Texas Capital Bank</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Diego Patino</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Executive Director, Senior Private Client Advisor</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr"/>
+      <c r="F23" s="7" t="inlineStr"/>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Own SEC-registered RIA</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Leads a specialist team for HNW families.</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>https://texascapitalbank.com/private-bank/meet-our-advisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Texas Capital Bank</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Joseph Gallardo</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Vice President, Private Client Advisor</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr"/>
+      <c r="F24" s="7" t="inlineStr"/>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Own SEC-registered RIA</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Primary relationship contact.</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>https://texascapitalbank.com/private-bank/meet-our-advisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Texas Capital Bank</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Annie Williams Cozad</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Vice President, Private Client Advisor</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr"/>
+      <c r="F25" s="7" t="inlineStr"/>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Own SEC-registered RIA</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr"/>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>https://texascapitalbank.com/private-bank/meet-our-advisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Texas Regional Bank</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Trey Willerson</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Chief Investment Officer</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Houston region</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr"/>
+      <c r="F26" s="7" t="inlineStr"/>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Own SEC-registered RIA</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>BEST TIMING IN TEXAS. A brand-new division that just hired a CIO is actively setting its investment process.</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>https://trb.bank/wealth-management/trust-wealth-team/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Texas Regional Bank</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Joshua Flores</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Chief Fiduciary Officer</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Houston region</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr"/>
+      <c r="F27" s="7" t="inlineStr"/>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Own SEC-registered RIA</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Trust side lead.</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>https://trb.bank/wealth-management/trust-wealth-team/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Texas Regional Bank</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Brian Cafferky</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Chief Operating Officer</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Houston region</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr"/>
+      <c r="F28" s="7" t="inlineStr"/>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Own SEC-registered RIA</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr"/>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>https://trb.bank/wealth-management/trust-wealth-team/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Texas Regional Bank</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Peyton Stamper</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Client Advisor</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Houston region</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr"/>
+      <c r="F29" s="7" t="inlineStr"/>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Own SEC-registered RIA</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr"/>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>https://trb.bank/wealth-management/trust-wealth-team/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Frost Bank</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Laurie Wieters</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Senior Vice President, Wealth Advisor</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>888-268-9202</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr"/>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Own BD + RIA (Frost)</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Largest self-contained wealth stack in Texas. Frost runs its OWN mutual funds, so proprietary product is a live issue here.</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>https://www.frostbank.com/personal/investments/trust-estate-planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Frost Bank</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Ashley Ferguson, CWS</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Vice President, Wealth Advisor</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>San Antonio (110 Austin Hwy)</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>888-268-9202</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr"/>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Own BD + RIA (Frost)</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr"/>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>https://www.frostbank.com/personal/investments/trust-estate-planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Jefferson Bank</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Todd Brockwell</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Leads 1900 Wealth</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>210-736-7600</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr"/>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>1900 Wealth is wholly owned by Jefferson Bank and runs independently.</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>https://1900wealth.com/trust-services/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Jefferson Bank</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Shawn Hughes, J.D.</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Division President of Trust</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>210-736-7600</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr"/>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>20 yrs probate/estates/guardianship law plus 8 yrs banking. Bench includes CFPs, CFAs, ex-pension managers, a Big Four tax specialist.</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>https://1900wealth.com/trust-services/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>First Financial Bank</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Grant Seabourne, CFP, CTFA</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Trust and estate planning</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Abilene</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>325-627-7100</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr"/>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary AND a separate Raymond James program</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>CTFA marks him trust-side. NOTE: First Financial has TWO channels - in-house trust AND First Financial Investment Advisors on Raymond James.</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>https://ffin.com/wealth-management/markets/abilene-office</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>First Financial Bank</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Zach Reyes</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Recently promoted</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Abilene</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>325-627-7100</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr"/>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>https://ffin.com/wealth-management/markets/abilene-office</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>First Financial Bank</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Kiley Hembree</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Recently promoted</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Abilene</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>325-627-7100</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr"/>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr"/>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>https://ffin.com/wealth-management/markets/abilene-office</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>First Financial Bank</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Joseph Craig</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Recently promoted</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Abilene</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>325-627-7100</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr"/>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>In-house trust / fiduciary</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr"/>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>https://ffin.com/wealth-management/markets/abilene-office</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Comerica</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>David Camp</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Private Banking Advisor</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Dallas (8225 Preston Rd)</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>877-888-0958</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>In-house private wealth</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr"/>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>https://www.comerica.com/wealth-management/investing/advisor-directory.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Comerica</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Jana Calongne</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Wealth Advisor</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Houston (2 Riverway, 14th Fl)</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>877-888-0958</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr"/>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>In-house private wealth</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr"/>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>https://www.comerica.com/wealth-management/investing/advisor-directory.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Comerica</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Janelle Walker</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Comerica insights contributor</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>877-888-0958</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr"/>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>In-house private wealth</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Role not confirmed as advisory.</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>https://www.comerica.com/wealth-management/investing/advisor-directory.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>Named people:</t>
+        </is>
+      </c>
+      <c r="B42" s="8">
+        <f>COUNTA(B5:B40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>With a direct phone:</t>
+        </is>
+      </c>
+      <c r="B43" s="8">
+        <f>COUNTIF(E5:E40,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="C43" s="8">
+        <f>COUNTIF(F5:F40,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>&lt;- with an email</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="44" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>NO CRD WAS CAPTURED FOR ANY TEXAS ADVISOR. FINRA BrokerCheck, SEC IAPD and FDIC were all blocked from this environment, and bank sites could not be fetched. Every name here came from web search of bank pages, Raymond James program pages and press releases. Registration status, tenure and disclosure history are UNVERIFIED for all 32 people. Run a real BrokerCheck lookup before any call.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:I40"/>
+  <mergeCells count="1">
+    <mergeCell ref="A45:I45"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1695,7 +3307,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>